<commit_message>
listini serie: S140 raggruppata per sigla, montante slim / soglia ribassata / lato anta come varianti
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YMK4dVsJMS4SCsnwzeiU3b
</commit_message>
<xml_diff>
--- a/listini-serie/dist/Listini_D67.xlsx
+++ b/listini-serie/dist/Listini_D67.xlsx
@@ -461,7 +461,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>LISTINI A GRIGLIA — AluK D67 — IWG 67ID (porte) — SENZA VETRO — prezzi di vendita in €, IVA esclusa — 14/09/2026</t>
+          <t>LISTINI A GRIGLIA — AluK D67 — IWG 67ID (porte) — SENZA VETRO — prezzi di vendita in €, IVA esclusa — 15/09/2026</t>
         </is>
       </c>
     </row>
@@ -1265,7 +1265,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Prezzi di listino in €, IVA esclusa, senza vetro. Ore manodopera 6.0 h. Generato il 14/09/2026.</t>
+          <t>Prezzi di listino in €, IVA esclusa, senza vetro. Ore manodopera 6.0 h. Generato il 15/09/2026.</t>
         </is>
       </c>
     </row>
@@ -1513,7 +1513,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Prezzi di listino in €, IVA esclusa, senza vetro. Ore manodopera 6.0 h. Generato il 14/09/2026.</t>
+          <t>Prezzi di listino in €, IVA esclusa, senza vetro. Ore manodopera 6.0 h. Generato il 15/09/2026.</t>
         </is>
       </c>
     </row>
@@ -1861,7 +1861,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Prezzi di listino in €, IVA esclusa, senza vetro. Ore manodopera 10.0 h. Generato il 14/09/2026.</t>
+          <t>Prezzi di listino in €, IVA esclusa, senza vetro. Ore manodopera 10.0 h. Generato il 15/09/2026.</t>
         </is>
       </c>
     </row>
@@ -2209,7 +2209,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Prezzi di listino in €, IVA esclusa, senza vetro. Ore manodopera 10.0 h. Generato il 14/09/2026.</t>
+          <t>Prezzi di listino in €, IVA esclusa, senza vetro. Ore manodopera 10.0 h. Generato il 15/09/2026.</t>
         </is>
       </c>
     </row>
@@ -2557,7 +2557,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Prezzi di listino in €, IVA esclusa, senza vetro. Ore manodopera 10.0 h. Generato il 14/09/2026.</t>
+          <t>Prezzi di listino in €, IVA esclusa, senza vetro. Ore manodopera 10.0 h. Generato il 15/09/2026.</t>
         </is>
       </c>
     </row>
@@ -2905,7 +2905,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Prezzi di listino in €, IVA esclusa, senza vetro. Ore manodopera 10.0 h. Generato il 14/09/2026.</t>
+          <t>Prezzi di listino in €, IVA esclusa, senza vetro. Ore manodopera 10.0 h. Generato il 15/09/2026.</t>
         </is>
       </c>
     </row>
@@ -3153,7 +3153,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Prezzi di listino in €, IVA esclusa, senza vetro. Ore manodopera 6.0 h. Generato il 14/09/2026.</t>
+          <t>Prezzi di listino in €, IVA esclusa, senza vetro. Ore manodopera 6.0 h. Generato il 15/09/2026.</t>
         </is>
       </c>
     </row>
@@ -3401,7 +3401,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Prezzi di listino in €, IVA esclusa, senza vetro. Ore manodopera 6.0 h. Generato il 14/09/2026.</t>
+          <t>Prezzi di listino in €, IVA esclusa, senza vetro. Ore manodopera 6.0 h. Generato il 15/09/2026.</t>
         </is>
       </c>
     </row>
@@ -3649,7 +3649,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Prezzi di listino in €, IVA esclusa, senza vetro. Ore manodopera 6.0 h. Generato il 14/09/2026.</t>
+          <t>Prezzi di listino in €, IVA esclusa, senza vetro. Ore manodopera 6.0 h. Generato il 15/09/2026.</t>
         </is>
       </c>
     </row>
@@ -3997,7 +3997,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Prezzi di listino in €, IVA esclusa, senza vetro. Ore manodopera 10.0 h. Generato il 14/09/2026.</t>
+          <t>Prezzi di listino in €, IVA esclusa, senza vetro. Ore manodopera 10.0 h. Generato il 15/09/2026.</t>
         </is>
       </c>
     </row>
@@ -4345,7 +4345,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Prezzi di listino in €, IVA esclusa, senza vetro. Ore manodopera 10.0 h. Generato il 14/09/2026.</t>
+          <t>Prezzi di listino in €, IVA esclusa, senza vetro. Ore manodopera 10.0 h. Generato il 15/09/2026.</t>
         </is>
       </c>
     </row>
@@ -4693,7 +4693,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Prezzi di listino in €, IVA esclusa, senza vetro. Ore manodopera 10.0 h. Generato il 14/09/2026.</t>
+          <t>Prezzi di listino in €, IVA esclusa, senza vetro. Ore manodopera 10.0 h. Generato il 15/09/2026.</t>
         </is>
       </c>
     </row>
@@ -4941,7 +4941,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Prezzi di listino in €, IVA esclusa, senza vetro. Ore manodopera 6.0 h. Generato il 14/09/2026.</t>
+          <t>Prezzi di listino in €, IVA esclusa, senza vetro. Ore manodopera 6.0 h. Generato il 15/09/2026.</t>
         </is>
       </c>
     </row>
@@ -5189,7 +5189,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Prezzi di listino in €, IVA esclusa, senza vetro. Ore manodopera 6.0 h. Generato il 14/09/2026.</t>
+          <t>Prezzi di listino in €, IVA esclusa, senza vetro. Ore manodopera 6.0 h. Generato il 15/09/2026.</t>
         </is>
       </c>
     </row>

</xml_diff>